<commit_message>
Add seller/agent contacts for Punta Esmeralda catalog
- agents-contacts.md: structured contacts for all sources selling Punta
  Esmeralda apartments (developer sales, Leona Raíces, Terraquea, RE/MAX
  Oceanside, Pura Vida, Jaco Real Estate CR) with phones, WhatsApp, email,
  and which unit codes each handles.
- build_table.py: add contact_phone / contact_email columns, auto-filled
  per source; regenerate CSV + XLSX (now 22 columns).
- README.md: reference agents-contacts.md and the new columns.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R9fLEGgD2qREshpfgmfEcD
</commit_message>
<xml_diff>
--- a/punta-esmeralda/punta-esmeralda-apartments.xlsx
+++ b/punta-esmeralda/punta-esmeralda-apartments.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Легенда" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Apartamentos'!$A$1:$T$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Apartamentos'!$A$1:$V$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -527,8 +527,10 @@
     <col width="11" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
     <col width="50" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="60" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="28" customWidth="1" min="21" max="21"/>
+    <col width="60" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -629,6 +631,16 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>contact_phone</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>contact_email</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
           <t>notes</t>
         </is>
       </c>
@@ -715,6 +727,16 @@
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
+          <t>+506 8810-4103</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>ventaspl@puntaesmeraldacr.com</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
           <t>Данные из флаера пользователя. Torre 4 Punta Esmeralda, Modelo A, vista bosque, cocina/sala/bodega/balcón/1 parqueo.</t>
         </is>
       </c>
@@ -797,6 +819,16 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
+          <t>+506 8810-4103</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>ventaspl@puntaesmeraldacr.com</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
           <t>Цена по запросу. Modelo A, cocina equipada, balcón vista bosque. Площадь оценочно ~61 м² (модель A).</t>
         </is>
       </c>
@@ -879,6 +911,16 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
+          <t>+506 8810-4103</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>ventaspl@puntaesmeraldacr.com</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
           <t>Цена по запросу. Vista bosque/mar, A/C completo, storage, parking, balcón.</t>
         </is>
       </c>
@@ -960,6 +1002,16 @@
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>+506 8810-4103</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>ventaspl@puntaesmeraldacr.com</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr">
         <is>
           <t>Цена по запросу. Balcón grande con vista al bosque.</t>
         </is>
@@ -1017,6 +1069,16 @@
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
+          <t>+506 4052-5777 / +506 8538-9249</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>info@terraquea.com</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
           <t>Vista al bosque. Точные спальни/площадь не указаны в открытом доступе.</t>
         </is>
       </c>
@@ -1090,6 +1152,16 @@
         </is>
       </c>
       <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>+506 4052-5777 / +506 8538-9249</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>info@terraquea.com</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
         <is>
           <t>Piso 5, llave en mano. Mantenimiento ~$210/мес.</t>
         </is>
@@ -1156,6 +1228,16 @@
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>+506 4052-5777 / +506 8538-9249</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>info@terraquea.com</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr">
         <is>
           <t>Piso 19, vista panorámica a la montaña. Mantenimiento ~$260/мес.</t>
         </is>
@@ -1224,6 +1306,16 @@
         </is>
       </c>
       <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>+506 4052-5777 / +506 8538-9249</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>info@terraquea.com</t>
+        </is>
+      </c>
+      <c r="V9" s="2" t="inlineStr">
         <is>
           <t>100% amueblado, piso 10 Torre 3, vista al mar.</t>
         </is>
@@ -1281,6 +1373,16 @@
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
+          <t>+506 4052-5777 / +506 8538-9249</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>info@terraquea.com</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
           <t>Condominio Punta Esmeralda, vista al bosque (код Terraquea 125574).</t>
         </is>
       </c>
@@ -1352,6 +1454,12 @@
         </is>
       </c>
       <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>+506 2643-4005 / +1 714-369-8263</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr"/>
+      <c r="V11" s="2" t="inlineStr">
         <is>
           <t>Fully titled, turnkey amueblado, vista parcial al mar, pasos de Playa Mantas. Цена по запросу.</t>
         </is>
@@ -1403,7 +1511,9 @@
           <t>Jaco Realty</t>
         </is>
       </c>
-      <c r="T12" s="2" t="inlineStr">
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr"/>
+      <c r="V12" s="2" t="inlineStr">
         <is>
           <t>Цена ~$285,000 (по видео Terraquea/Facebook).</t>
         </is>
@@ -1457,6 +1567,12 @@
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
+          <t>+506 4702-4000 / +506 2637-1919</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr"/>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
           <t>3 спальни, верхний этаж (top floor). Цена по запросу.</t>
         </is>
       </c>
@@ -1519,6 +1635,16 @@
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
+          <t>+506 4052-5777 / +506 8538-9249</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>info@terraquea.com</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
           <t>Piso 5, vista al mar. Крупный юнит ~140 м². Цена по запросу.</t>
         </is>
       </c>
@@ -1589,6 +1715,16 @@
       <c r="S15" s="6" t="inlineStr"/>
       <c r="T15" s="6" t="inlineStr">
         <is>
+          <t>+506 8922-5050</t>
+        </is>
+      </c>
+      <c r="U15" s="6" t="inlineStr">
+        <is>
+          <t>ventaspl@puntaesmeraldacr.com</t>
+        </is>
+      </c>
+      <c r="V15" s="6" t="inlineStr">
+        <is>
           <t>Типовая модель A: 2 сп./1 с/у, ~61-65 м², вид на лес. Типичная перепродажа $200-220k.</t>
         </is>
       </c>
@@ -1659,6 +1795,16 @@
       <c r="S16" s="6" t="inlineStr"/>
       <c r="T16" s="6" t="inlineStr">
         <is>
+          <t>+506 8922-5050</t>
+        </is>
+      </c>
+      <c r="U16" s="6" t="inlineStr">
+        <is>
+          <t>ventaspl@puntaesmeraldacr.com</t>
+        </is>
+      </c>
+      <c r="V16" s="6" t="inlineStr">
+        <is>
           <t>Типовая модель B: 2-3 сп./2 с/у, ~83-102 м², вид на море/горы. Типичная цена $260-295k.</t>
         </is>
       </c>
@@ -1728,6 +1874,16 @@
       </c>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr">
+        <is>
+          <t>+506 8922-5050</t>
+        </is>
+      </c>
+      <c r="U17" s="6" t="inlineStr">
+        <is>
+          <t>ventaspl@puntaesmeraldacr.com</t>
+        </is>
+      </c>
+      <c r="V17" s="6" t="inlineStr">
         <is>
           <t>Объединённый/премиум юнит: ~140 м², вид на океан, верхние этажи.</t>
         </is>
@@ -1793,6 +1949,16 @@
       </c>
       <c r="T18" s="9" t="inlineStr">
         <is>
+          <t>+506 8922-5050</t>
+        </is>
+      </c>
+      <c r="U18" s="9" t="inlineStr">
+        <is>
+          <t>ventaspl@puntaesmeraldacr.com</t>
+        </is>
+      </c>
+      <c r="V18" s="9" t="inlineStr">
+        <is>
           <t>Torre 1 распродана застройщиком. $107k — стартовая цена застройщика (2 сп.), НЕ цена конкретной сделки. Точные цены сделок в Коста-Рике не публичны.</t>
         </is>
       </c>
@@ -1857,6 +2023,16 @@
       </c>
       <c r="T19" s="9" t="inlineStr">
         <is>
+          <t>+506 8922-5050</t>
+        </is>
+      </c>
+      <c r="U19" s="9" t="inlineStr">
+        <is>
+          <t>ventaspl@puntaesmeraldacr.com</t>
+        </is>
+      </c>
+      <c r="V19" s="9" t="inlineStr">
+        <is>
           <t>«Última Torre 2» — оставались последние юниты. $110k — оценка стартовой цены застройщика, не цена сделки.</t>
         </is>
       </c>
@@ -1921,12 +2097,22 @@
       </c>
       <c r="T20" s="9" t="inlineStr">
         <is>
+          <t>+506 8922-5050</t>
+        </is>
+      </c>
+      <c r="U20" s="9" t="inlineStr">
+        <is>
+          <t>ventaspl@puntaesmeraldacr.com</t>
+        </is>
+      </c>
+      <c r="V20" s="9" t="inlineStr">
+        <is>
           <t>Torre 3 сдана 06/2023, первичные продажи в основном закрыты. На вторичке сейчас $260k+ (см. T3-13-04A, TQ-131516). $150k — оценка первички, не цена сделки.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T20"/>
+  <autoFilter ref="A1:V20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1937,7 +2123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2204,45 +2390,69 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>Контакт агента/застройщика</t>
+          <t>Имя агента / контактное лицо</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>contact_phone</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>Примечания, оговорки по достоверности</t>
+          <t>Телефон / WhatsApp агентства (см. agents-contacts.md)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr"/>
-      <c r="B25" s="13" t="inlineStr"/>
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>contact_email</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Email агентства / отдела продаж</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Примечания, оговорки по достоверности</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr"/>
+      <c r="B27" s="13" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
           <t>ВАЖНО про цены продаж</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Индивидуальные цены сделок в Коста-Рике публично не раскрываются (нет публичного API; суммы в Registro Nacional часто занижены). Строки sold показывают оценку первичных цен застройщика, а не конкретные сделки.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>Как сортировать</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Excel: вкладка 'Данные' -&gt; стрелка в шапке столбца. Google Sheets: Данные -&gt; Создать фильтр.</t>
         </is>

</xml_diff>